<commit_message>
Update of the audio files and improved split
</commit_message>
<xml_diff>
--- a/original/de/german_talking_clock_audio_list.xlsx
+++ b/original/de/german_talking_clock_audio_list.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>Language</t>
   </si>
@@ -47,6 +47,150 @@
   </si>
   <si>
     <t>mitternacht</t>
+  </si>
+  <si>
+    <t>0h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist mitternacht</t>
+  </si>
+  <si>
+    <t>1h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist eine uhr</t>
+  </si>
+  <si>
+    <t>2h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 2 uhr</t>
+  </si>
+  <si>
+    <t>3h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 3 uhr</t>
+  </si>
+  <si>
+    <t>4h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 4 uhr</t>
+  </si>
+  <si>
+    <t>5h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 5 uhr</t>
+  </si>
+  <si>
+    <t>6h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 6 uhr</t>
+  </si>
+  <si>
+    <t>7h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 7 uhr</t>
+  </si>
+  <si>
+    <t>8h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 8 uhr</t>
+  </si>
+  <si>
+    <t>9h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 9 uhr</t>
+  </si>
+  <si>
+    <t>10h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 10 uhr</t>
+  </si>
+  <si>
+    <t>11h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 11 uhr</t>
+  </si>
+  <si>
+    <t>12h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 12 uhr</t>
+  </si>
+  <si>
+    <t>13h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 13 uhr</t>
+  </si>
+  <si>
+    <t>14h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 14 uhr</t>
+  </si>
+  <si>
+    <t>15h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 15 uhr</t>
+  </si>
+  <si>
+    <t>16h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 16 uhr</t>
+  </si>
+  <si>
+    <t>17h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 17 uhr</t>
+  </si>
+  <si>
+    <t>18h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 18 uhr</t>
+  </si>
+  <si>
+    <t>19h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 19 uhr</t>
+  </si>
+  <si>
+    <t>20h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 20 uhr</t>
+  </si>
+  <si>
+    <t>21h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 21 uhr</t>
+  </si>
+  <si>
+    <t>22h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 22 uhr</t>
+  </si>
+  <si>
+    <t>23h.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Es ist 23 uhr</t>
   </si>
   <si>
     <t>English</t>
@@ -157,7 +301,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -176,6 +320,9 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -708,348 +855,324 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="str">
-        <f t="shared" ref="B5:B9" si="0">_xlfn.CONCAT(C5,".mp3")</f>
-        <v>1.mp3</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1</v>
+      <c r="B5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="15">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1" t="str">
+      <c r="B6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="15">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" ht="15">
+      <c r="A8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" ht="15">
+      <c r="A9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" ht="15">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" ht="15">
+      <c r="A11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" ht="15">
+      <c r="A12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" ht="15">
+      <c r="A13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" ht="15">
+      <c r="A14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" ht="15">
+      <c r="A15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" ht="15">
+      <c r="A16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" ht="15">
+      <c r="A17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" ht="15">
+      <c r="A18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" ht="15">
+      <c r="A19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" ht="15">
+      <c r="A20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" ht="15">
+      <c r="A21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" ht="15">
+      <c r="A22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" ht="15">
+      <c r="A23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" ht="15">
+      <c r="A24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" ht="15">
+      <c r="A25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" ht="15">
+      <c r="A26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" ht="15">
+      <c r="A27" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" ht="15">
+      <c r="A28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" ht="15">
+      <c r="A29" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="1" t="str">
+        <f t="shared" ref="B29:B33" si="0">_xlfn.CONCAT(C29,".mp3")</f>
+        <v>1.mp3</v>
+      </c>
+      <c r="C29" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" ht="15">
+      <c r="A30" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="1" t="str">
         <f t="shared" si="0"/>
         <v>2.mp3</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C30" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="15">
-      <c r="A7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="1" t="str">
+    <row r="31" ht="15">
+      <c r="A31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="1" t="str">
         <f t="shared" si="0"/>
         <v>3.mp3</v>
       </c>
-      <c r="C7" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" ht="15">
-      <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="1" t="str">
+      <c r="C31" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" ht="15">
+      <c r="A32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" s="1" t="str">
         <f t="shared" si="0"/>
         <v>4.mp3</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C32" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="9" ht="15">
-      <c r="A9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="str">
+    <row r="33" ht="15">
+      <c r="A33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="1" t="str">
         <f t="shared" si="0"/>
         <v>5.mp3</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C33" s="2">
         <v>5</v>
-      </c>
-    </row>
-    <row r="10" ht="15">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="str">
-        <f t="shared" ref="B10:B63" si="1">_xlfn.CONCAT(C10,".mp3")</f>
-        <v>6.mp3</v>
-      </c>
-      <c r="C10" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" ht="15">
-      <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>7.mp3</v>
-      </c>
-      <c r="C11" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" ht="15">
-      <c r="A12" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>8.mp3</v>
-      </c>
-      <c r="C12" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" ht="15">
-      <c r="A13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>9.mp3</v>
-      </c>
-      <c r="C13" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" ht="15">
-      <c r="A14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>10.mp3</v>
-      </c>
-      <c r="C14" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" ht="15">
-      <c r="A15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>11.mp3</v>
-      </c>
-      <c r="C15" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" ht="15">
-      <c r="A16" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>12.mp3</v>
-      </c>
-      <c r="C16" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" ht="15">
-      <c r="A17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>13.mp3</v>
-      </c>
-      <c r="C17" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" ht="15">
-      <c r="A18" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>14.mp3</v>
-      </c>
-      <c r="C18" s="2">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" ht="15">
-      <c r="A19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>15.mp3</v>
-      </c>
-      <c r="C19" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" ht="15">
-      <c r="A20" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>16.mp3</v>
-      </c>
-      <c r="C20" s="2">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" ht="15">
-      <c r="A21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>17.mp3</v>
-      </c>
-      <c r="C21" s="2">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" ht="15">
-      <c r="A22" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>18.mp3</v>
-      </c>
-      <c r="C22" s="2">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" ht="15">
-      <c r="A23" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B23" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>19.mp3</v>
-      </c>
-      <c r="C23" s="2">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" ht="15">
-      <c r="A24" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>20.mp3</v>
-      </c>
-      <c r="C24" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" ht="15">
-      <c r="A25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>21.mp3</v>
-      </c>
-      <c r="C25" s="2">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" ht="15">
-      <c r="A26" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>22.mp3</v>
-      </c>
-      <c r="C26" s="2">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" ht="15">
-      <c r="A27" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>23.mp3</v>
-      </c>
-      <c r="C27" s="2">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" ht="15">
-      <c r="A28" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>24.mp3</v>
-      </c>
-      <c r="C28" s="2">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" ht="15">
-      <c r="A29" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>25.mp3</v>
-      </c>
-      <c r="C29" s="2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" ht="15">
-      <c r="A30" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>26.mp3</v>
-      </c>
-      <c r="C30" s="2">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" ht="15">
-      <c r="A31" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>27.mp3</v>
-      </c>
-      <c r="C31" s="2">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="32" ht="15">
-      <c r="A32" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>28.mp3</v>
-      </c>
-      <c r="C32" s="2">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="33" ht="15">
-      <c r="A33" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>29.mp3</v>
-      </c>
-      <c r="C33" s="2">
-        <v>29</v>
       </c>
     </row>
     <row r="34" ht="15">
@@ -1057,11 +1180,11 @@
         <v>3</v>
       </c>
       <c r="B34" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>30.mp3</v>
+        <f t="shared" ref="B34:B87" si="1">_xlfn.CONCAT(C34,".mp3")</f>
+        <v>6.mp3</v>
       </c>
       <c r="C34" s="2">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" ht="15">
@@ -1070,10 +1193,10 @@
       </c>
       <c r="B35" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>31.mp3</v>
+        <v>7.mp3</v>
       </c>
       <c r="C35" s="2">
-        <v>31</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" ht="15">
@@ -1082,10 +1205,10 @@
       </c>
       <c r="B36" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>32.mp3</v>
+        <v>8.mp3</v>
       </c>
       <c r="C36" s="2">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" ht="15">
@@ -1094,10 +1217,10 @@
       </c>
       <c r="B37" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>33.mp3</v>
+        <v>9.mp3</v>
       </c>
       <c r="C37" s="2">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" ht="15">
@@ -1106,10 +1229,10 @@
       </c>
       <c r="B38" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>34.mp3</v>
+        <v>10.mp3</v>
       </c>
       <c r="C38" s="2">
-        <v>34</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" ht="15">
@@ -1118,10 +1241,10 @@
       </c>
       <c r="B39" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>35.mp3</v>
+        <v>11.mp3</v>
       </c>
       <c r="C39" s="2">
-        <v>35</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40" ht="15">
@@ -1130,10 +1253,10 @@
       </c>
       <c r="B40" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>36.mp3</v>
+        <v>12.mp3</v>
       </c>
       <c r="C40" s="2">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" ht="15">
@@ -1142,10 +1265,10 @@
       </c>
       <c r="B41" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>37.mp3</v>
+        <v>13.mp3</v>
       </c>
       <c r="C41" s="2">
-        <v>37</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" ht="15">
@@ -1154,10 +1277,10 @@
       </c>
       <c r="B42" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>38.mp3</v>
+        <v>14.mp3</v>
       </c>
       <c r="C42" s="2">
-        <v>38</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" ht="15">
@@ -1166,10 +1289,10 @@
       </c>
       <c r="B43" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>39.mp3</v>
+        <v>15.mp3</v>
       </c>
       <c r="C43" s="2">
-        <v>39</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44" ht="15">
@@ -1178,10 +1301,10 @@
       </c>
       <c r="B44" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>40.mp3</v>
+        <v>16.mp3</v>
       </c>
       <c r="C44" s="2">
-        <v>40</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" ht="15">
@@ -1190,10 +1313,10 @@
       </c>
       <c r="B45" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>41.mp3</v>
+        <v>17.mp3</v>
       </c>
       <c r="C45" s="2">
-        <v>41</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" ht="15">
@@ -1202,10 +1325,10 @@
       </c>
       <c r="B46" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>42.mp3</v>
+        <v>18.mp3</v>
       </c>
       <c r="C46" s="2">
-        <v>42</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47" ht="15">
@@ -1214,10 +1337,10 @@
       </c>
       <c r="B47" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>43.mp3</v>
+        <v>19.mp3</v>
       </c>
       <c r="C47" s="2">
-        <v>43</v>
+        <v>19</v>
       </c>
     </row>
     <row r="48" ht="15">
@@ -1226,10 +1349,10 @@
       </c>
       <c r="B48" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>44.mp3</v>
+        <v>20.mp3</v>
       </c>
       <c r="C48" s="2">
-        <v>44</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" ht="15">
@@ -1238,10 +1361,10 @@
       </c>
       <c r="B49" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>45.mp3</v>
+        <v>21.mp3</v>
       </c>
       <c r="C49" s="2">
-        <v>45</v>
+        <v>21</v>
       </c>
     </row>
     <row r="50" ht="15">
@@ -1250,10 +1373,10 @@
       </c>
       <c r="B50" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>46.mp3</v>
+        <v>22.mp3</v>
       </c>
       <c r="C50" s="2">
-        <v>46</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51" ht="15">
@@ -1262,10 +1385,10 @@
       </c>
       <c r="B51" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>47.mp3</v>
+        <v>23.mp3</v>
       </c>
       <c r="C51" s="2">
-        <v>47</v>
+        <v>23</v>
       </c>
     </row>
     <row r="52" ht="15">
@@ -1274,10 +1397,10 @@
       </c>
       <c r="B52" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>48.mp3</v>
+        <v>24.mp3</v>
       </c>
       <c r="C52" s="2">
-        <v>48</v>
+        <v>24</v>
       </c>
     </row>
     <row r="53" ht="15">
@@ -1286,10 +1409,10 @@
       </c>
       <c r="B53" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>49.mp3</v>
+        <v>25.mp3</v>
       </c>
       <c r="C53" s="2">
-        <v>49</v>
+        <v>25</v>
       </c>
     </row>
     <row r="54" ht="15">
@@ -1298,10 +1421,10 @@
       </c>
       <c r="B54" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>50.mp3</v>
+        <v>26.mp3</v>
       </c>
       <c r="C54" s="2">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55" ht="15">
@@ -1310,10 +1433,10 @@
       </c>
       <c r="B55" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>51.mp3</v>
+        <v>27.mp3</v>
       </c>
       <c r="C55" s="2">
-        <v>51</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" ht="15">
@@ -1322,10 +1445,10 @@
       </c>
       <c r="B56" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>52.mp3</v>
+        <v>28.mp3</v>
       </c>
       <c r="C56" s="2">
-        <v>52</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57" ht="15">
@@ -1334,10 +1457,10 @@
       </c>
       <c r="B57" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>53.mp3</v>
+        <v>29.mp3</v>
       </c>
       <c r="C57" s="2">
-        <v>53</v>
+        <v>29</v>
       </c>
     </row>
     <row r="58" ht="15">
@@ -1346,10 +1469,10 @@
       </c>
       <c r="B58" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>54.mp3</v>
+        <v>30.mp3</v>
       </c>
       <c r="C58" s="2">
-        <v>54</v>
+        <v>30</v>
       </c>
     </row>
     <row r="59" ht="15">
@@ -1358,10 +1481,10 @@
       </c>
       <c r="B59" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>55.mp3</v>
+        <v>31.mp3</v>
       </c>
       <c r="C59" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60" ht="15">
@@ -1370,10 +1493,10 @@
       </c>
       <c r="B60" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>56.mp3</v>
+        <v>32.mp3</v>
       </c>
       <c r="C60" s="2">
-        <v>56</v>
+        <v>32</v>
       </c>
     </row>
     <row r="61" ht="15">
@@ -1382,10 +1505,10 @@
       </c>
       <c r="B61" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>57.mp3</v>
+        <v>33.mp3</v>
       </c>
       <c r="C61" s="2">
-        <v>57</v>
+        <v>33</v>
       </c>
     </row>
     <row r="62" ht="15">
@@ -1394,10 +1517,10 @@
       </c>
       <c r="B62" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>58.mp3</v>
+        <v>34.mp3</v>
       </c>
       <c r="C62" s="2">
-        <v>58</v>
+        <v>34</v>
       </c>
     </row>
     <row r="63" ht="15">
@@ -1406,238 +1529,522 @@
       </c>
       <c r="B63" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>59.mp3</v>
+        <v>35.mp3</v>
       </c>
       <c r="C63" s="2">
-        <v>59</v>
+        <v>35</v>
       </c>
     </row>
     <row r="64" ht="15">
       <c r="A64" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>12</v>
+        <v>3</v>
+      </c>
+      <c r="B64" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>36.mp3</v>
+      </c>
+      <c r="C64" s="2">
+        <v>36</v>
       </c>
     </row>
     <row r="65" ht="15">
       <c r="A65" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>14</v>
+        <v>3</v>
+      </c>
+      <c r="B65" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>37.mp3</v>
+      </c>
+      <c r="C65" s="2">
+        <v>37</v>
       </c>
     </row>
     <row r="66" ht="15">
       <c r="A66" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>16</v>
+        <v>3</v>
+      </c>
+      <c r="B66" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>38.mp3</v>
+      </c>
+      <c r="C66" s="2">
+        <v>38</v>
       </c>
     </row>
     <row r="67" ht="15">
       <c r="A67" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>18</v>
+        <v>3</v>
+      </c>
+      <c r="B67" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>39.mp3</v>
+      </c>
+      <c r="C67" s="2">
+        <v>39</v>
       </c>
     </row>
     <row r="68" ht="15">
       <c r="A68" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>20</v>
+        <v>3</v>
+      </c>
+      <c r="B68" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>40.mp3</v>
+      </c>
+      <c r="C68" s="2">
+        <v>40</v>
       </c>
     </row>
     <row r="69" ht="15">
       <c r="A69" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B69" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>22</v>
+        <v>3</v>
+      </c>
+      <c r="B69" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>41.mp3</v>
+      </c>
+      <c r="C69" s="2">
+        <v>41</v>
       </c>
     </row>
     <row r="70" ht="15">
       <c r="A70" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>24</v>
+        <v>3</v>
+      </c>
+      <c r="B70" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>42.mp3</v>
+      </c>
+      <c r="C70" s="2">
+        <v>42</v>
       </c>
     </row>
     <row r="71" ht="15">
-      <c r="A71" s="1"/>
-      <c r="B71" s="1"/>
-      <c r="C71" s="2"/>
+      <c r="A71" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B71" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>43.mp3</v>
+      </c>
+      <c r="C71" s="2">
+        <v>43</v>
+      </c>
     </row>
     <row r="72" ht="15">
-      <c r="A72" s="1"/>
-      <c r="B72" s="1"/>
-      <c r="C72" s="2"/>
+      <c r="A72" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B72" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>44.mp3</v>
+      </c>
+      <c r="C72" s="2">
+        <v>44</v>
+      </c>
     </row>
     <row r="73" ht="15">
-      <c r="A73" s="1"/>
-      <c r="B73" s="1"/>
-      <c r="C73" s="2"/>
+      <c r="A73" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B73" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>45.mp3</v>
+      </c>
+      <c r="C73" s="2">
+        <v>45</v>
+      </c>
     </row>
     <row r="74" ht="15">
-      <c r="A74" s="1"/>
-      <c r="B74" s="1"/>
-      <c r="C74" s="2"/>
+      <c r="A74" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B74" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>46.mp3</v>
+      </c>
+      <c r="C74" s="2">
+        <v>46</v>
+      </c>
     </row>
     <row r="75" ht="15">
-      <c r="A75" s="1"/>
-      <c r="B75" s="1"/>
-      <c r="C75" s="2"/>
+      <c r="A75" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B75" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>47.mp3</v>
+      </c>
+      <c r="C75" s="2">
+        <v>47</v>
+      </c>
     </row>
     <row r="76" ht="15">
-      <c r="A76" s="1"/>
-      <c r="B76" s="1"/>
-      <c r="C76" s="2"/>
+      <c r="A76" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B76" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>48.mp3</v>
+      </c>
+      <c r="C76" s="2">
+        <v>48</v>
+      </c>
     </row>
     <row r="77" ht="15">
-      <c r="A77" s="1"/>
-      <c r="B77" s="1"/>
-      <c r="C77" s="2"/>
+      <c r="A77" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B77" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>49.mp3</v>
+      </c>
+      <c r="C77" s="2">
+        <v>49</v>
+      </c>
     </row>
     <row r="78" ht="15">
-      <c r="A78" s="1"/>
-      <c r="B78" s="1"/>
-      <c r="C78" s="2"/>
+      <c r="A78" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B78" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>50.mp3</v>
+      </c>
+      <c r="C78" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="79" ht="15">
-      <c r="A79" s="1"/>
-      <c r="B79" s="1"/>
-      <c r="C79" s="2"/>
+      <c r="A79" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B79" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>51.mp3</v>
+      </c>
+      <c r="C79" s="2">
+        <v>51</v>
+      </c>
     </row>
     <row r="80" ht="15">
-      <c r="A80" s="1"/>
-      <c r="B80" s="1"/>
-      <c r="C80" s="2"/>
+      <c r="A80" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B80" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>52.mp3</v>
+      </c>
+      <c r="C80" s="2">
+        <v>52</v>
+      </c>
     </row>
     <row r="81" ht="15">
-      <c r="A81" s="1"/>
-      <c r="B81" s="1"/>
-      <c r="C81" s="2"/>
+      <c r="A81" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B81" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>53.mp3</v>
+      </c>
+      <c r="C81" s="2">
+        <v>53</v>
+      </c>
     </row>
     <row r="82" ht="15">
-      <c r="A82" s="1"/>
-      <c r="B82" s="1"/>
-      <c r="C82" s="2"/>
+      <c r="A82" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B82" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>54.mp3</v>
+      </c>
+      <c r="C82" s="2">
+        <v>54</v>
+      </c>
     </row>
     <row r="83" ht="15">
-      <c r="A83" s="1"/>
-      <c r="B83" s="1"/>
-      <c r="C83" s="2"/>
+      <c r="A83" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B83" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>55.mp3</v>
+      </c>
+      <c r="C83" s="2">
+        <v>55</v>
+      </c>
     </row>
     <row r="84" ht="15">
-      <c r="A84" s="1"/>
-      <c r="B84" s="1"/>
-      <c r="C84" s="2"/>
+      <c r="A84" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B84" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>56.mp3</v>
+      </c>
+      <c r="C84" s="2">
+        <v>56</v>
+      </c>
     </row>
     <row r="85" ht="15">
-      <c r="A85" s="1"/>
-      <c r="B85" s="1"/>
-      <c r="C85" s="2"/>
+      <c r="A85" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B85" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>57.mp3</v>
+      </c>
+      <c r="C85" s="2">
+        <v>57</v>
+      </c>
     </row>
     <row r="86" ht="15">
-      <c r="A86" s="1"/>
-      <c r="B86" s="1"/>
-      <c r="C86" s="2"/>
+      <c r="A86" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B86" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>58.mp3</v>
+      </c>
+      <c r="C86" s="2">
+        <v>58</v>
+      </c>
     </row>
     <row r="87" ht="15">
-      <c r="A87" s="1"/>
-      <c r="B87" s="1"/>
-      <c r="C87" s="2"/>
+      <c r="A87" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B87" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>59.mp3</v>
+      </c>
+      <c r="C87" s="2">
+        <v>59</v>
+      </c>
     </row>
     <row r="88" ht="15">
-      <c r="A88" s="1"/>
-      <c r="B88" s="1"/>
-      <c r="C88" s="2"/>
+      <c r="A88" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="89" ht="15">
-      <c r="A89" s="1"/>
-      <c r="B89" s="1"/>
-      <c r="C89" s="2"/>
+      <c r="A89" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="90" ht="15">
-      <c r="A90" s="1"/>
-      <c r="B90" s="1"/>
-      <c r="C90" s="2"/>
+      <c r="A90" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="91" ht="15">
-      <c r="A91" s="1"/>
+      <c r="A91" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="92" ht="15">
-      <c r="A92" s="1"/>
+      <c r="A92" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="93" ht="15">
-      <c r="A93" s="1"/>
+      <c r="A93" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="94" ht="15">
-      <c r="A94" s="1"/>
+      <c r="A94" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="95" ht="15">
       <c r="A95" s="1"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="2"/>
     </row>
     <row r="96" ht="15">
       <c r="A96" s="1"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="2"/>
     </row>
     <row r="97" ht="15">
       <c r="A97" s="1"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="2"/>
     </row>
     <row r="98" ht="15">
       <c r="A98" s="1"/>
+      <c r="B98" s="1"/>
+      <c r="C98" s="2"/>
     </row>
     <row r="99" ht="15">
       <c r="A99" s="1"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="2"/>
     </row>
     <row r="100" ht="15">
       <c r="A100" s="1"/>
+      <c r="B100" s="1"/>
+      <c r="C100" s="2"/>
     </row>
     <row r="101" ht="15">
       <c r="A101" s="1"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="2"/>
     </row>
     <row r="102" ht="15">
       <c r="A102" s="1"/>
+      <c r="B102" s="1"/>
+      <c r="C102" s="2"/>
     </row>
     <row r="103" ht="15">
       <c r="A103" s="1"/>
+      <c r="B103" s="1"/>
+      <c r="C103" s="2"/>
     </row>
     <row r="104" ht="15">
       <c r="A104" s="1"/>
+      <c r="B104" s="1"/>
+      <c r="C104" s="2"/>
     </row>
     <row r="105" ht="15">
       <c r="A105" s="1"/>
-    </row>
-    <row r="1048573" ht="12.800000000000001"/>
-    <row r="1048574" ht="12.800000000000001"/>
-    <row r="1048575" ht="12.800000000000001"/>
-    <row r="1048576" ht="12.800000000000001"/>
+      <c r="B105" s="1"/>
+      <c r="C105" s="2"/>
+    </row>
+    <row r="106" ht="15">
+      <c r="A106" s="1"/>
+      <c r="B106" s="1"/>
+      <c r="C106" s="2"/>
+    </row>
+    <row r="107" ht="15">
+      <c r="A107" s="1"/>
+      <c r="B107" s="1"/>
+      <c r="C107" s="2"/>
+    </row>
+    <row r="108" ht="15">
+      <c r="A108" s="1"/>
+      <c r="B108" s="1"/>
+      <c r="C108" s="2"/>
+    </row>
+    <row r="109" ht="15">
+      <c r="A109" s="1"/>
+      <c r="B109" s="1"/>
+      <c r="C109" s="2"/>
+    </row>
+    <row r="110" ht="15">
+      <c r="A110" s="1"/>
+      <c r="B110" s="1"/>
+      <c r="C110" s="2"/>
+    </row>
+    <row r="111" ht="15">
+      <c r="A111" s="1"/>
+      <c r="B111" s="1"/>
+      <c r="C111" s="2"/>
+    </row>
+    <row r="112" ht="15">
+      <c r="A112" s="1"/>
+      <c r="B112" s="1"/>
+      <c r="C112" s="2"/>
+    </row>
+    <row r="113" ht="15">
+      <c r="A113" s="1"/>
+      <c r="B113" s="1"/>
+      <c r="C113" s="2"/>
+    </row>
+    <row r="114" ht="15">
+      <c r="A114" s="1"/>
+      <c r="B114" s="1"/>
+      <c r="C114" s="2"/>
+    </row>
+    <row r="115" ht="15">
+      <c r="A115" s="1"/>
+    </row>
+    <row r="116" ht="15">
+      <c r="A116" s="1"/>
+    </row>
+    <row r="117" ht="15">
+      <c r="A117" s="1"/>
+    </row>
+    <row r="118" ht="15">
+      <c r="A118" s="1"/>
+    </row>
+    <row r="119" ht="15">
+      <c r="A119" s="1"/>
+    </row>
+    <row r="120" ht="15">
+      <c r="A120" s="1"/>
+    </row>
+    <row r="121" ht="15">
+      <c r="A121" s="1"/>
+    </row>
+    <row r="122" ht="15">
+      <c r="A122" s="1"/>
+    </row>
+    <row r="123" ht="15">
+      <c r="A123" s="1"/>
+    </row>
+    <row r="124" ht="15">
+      <c r="A124" s="1"/>
+    </row>
+    <row r="125" ht="15">
+      <c r="A125" s="1"/>
+    </row>
+    <row r="126" ht="15">
+      <c r="A126" s="1"/>
+    </row>
+    <row r="127" ht="15">
+      <c r="A127" s="1"/>
+    </row>
+    <row r="128" ht="15">
+      <c r="A128" s="1"/>
+    </row>
+    <row r="129" ht="15">
+      <c r="A129" s="1"/>
+    </row>
   </sheetData>
   <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>

</xml_diff>